<commit_message>
Change of Cadarache for France
</commit_message>
<xml_diff>
--- a/2026 ATG at F4E Public Holidays.xlsx
+++ b/2026 ATG at F4E Public Holidays.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\carboed\Documents\Team Liason\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\carboed\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5A58F8-9E7B-4764-A74E-57C77B2088FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F337E668-F1D0-433F-8A62-50BB9D7DD2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{14DBFD9E-4591-4947-AA2F-CC76908940A1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{14DBFD9E-4591-4947-AA2F-CC76908940A1}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 PH" sheetId="1" r:id="rId1"/>
@@ -48,9 +48,6 @@
     <t>Cantabria</t>
   </si>
   <si>
-    <t>Cadarache</t>
-  </si>
-  <si>
     <t>Garching</t>
   </si>
   <si>
@@ -264,6 +261,9 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>France</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1044,7 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>0</v>
@@ -1056,19 +1056,19 @@
         <v>2</v>
       </c>
       <c r="E1" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>6</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -1076,28 +1076,28 @@
         <v>46023</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1105,30 +1105,30 @@
         <v>46024</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K3" s="6"/>
       <c r="L3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1137,21 +1137,21 @@
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K4" s="7"/>
       <c r="L4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1159,22 +1159,22 @@
         <v>46028</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -1187,7 +1187,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
@@ -1202,7 +1202,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
@@ -1217,7 +1217,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -1232,7 +1232,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -1243,21 +1243,21 @@
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1265,26 +1265,26 @@
         <v>46115</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1292,20 +1292,20 @@
         <v>46118</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="10"/>
       <c r="I12" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1318,7 +1318,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -1328,26 +1328,26 @@
         <v>46143</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1360,7 +1360,7 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -1375,7 +1375,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -1390,7 +1390,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -1403,7 +1403,7 @@
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1418,10 +1418,10 @@
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -1435,10 +1435,10 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -1449,15 +1449,15 @@
         <v>46167</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1470,7 +1470,7 @@
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
@@ -1490,7 +1490,7 @@
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1499,19 +1499,19 @@
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1525,7 +1525,7 @@
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I25" s="4"/>
     </row>
@@ -1540,7 +1540,7 @@
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I26" s="4"/>
     </row>
@@ -1549,11 +1549,11 @@
         <v>46197</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
@@ -1569,7 +1569,7 @@
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
       <c r="E28" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -1584,7 +1584,7 @@
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -1601,7 +1601,7 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
@@ -1613,7 +1613,7 @@
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
@@ -1631,7 +1631,7 @@
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
@@ -1641,7 +1641,7 @@
         <v>46276</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
@@ -1658,7 +1658,7 @@
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
@@ -1676,7 +1676,7 @@
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
@@ -1691,7 +1691,7 @@
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
@@ -1706,7 +1706,7 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
@@ -1716,7 +1716,7 @@
         <v>46289</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
@@ -1737,7 +1737,7 @@
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I39" s="4"/>
     </row>
@@ -1746,18 +1746,18 @@
         <v>46307</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
@@ -1787,7 +1787,7 @@
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
@@ -1800,7 +1800,7 @@
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
       <c r="E43" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
@@ -1817,7 +1817,7 @@
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
@@ -1833,7 +1833,7 @@
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I45" s="4"/>
     </row>
@@ -1843,19 +1843,19 @@
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -1863,22 +1863,22 @@
         <v>46364</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -1886,28 +1886,28 @@
         <v>46380</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -1915,28 +1915,28 @@
         <v>46381</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -1944,28 +1944,28 @@
         <v>46384</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -1973,28 +1973,28 @@
         <v>46385</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2002,28 +2002,28 @@
         <v>46386</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2031,28 +2031,28 @@
         <v>46387</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2075,251 +2075,251 @@
   <sheetData>
     <row r="1" spans="1:25">
       <c r="A1" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="Y1" t="s">
         <v>12</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="30" spans="11:11">
       <c r="K30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:12">
       <c r="A37" t="s">
+        <v>14</v>
+      </c>
+      <c r="K37" t="s">
         <v>15</v>
-      </c>
-      <c r="K37" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="39" spans="1:12">
       <c r="K39" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L39" s="13"/>
     </row>
     <row r="40" spans="1:12">
       <c r="K40" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L40" s="13"/>
     </row>
     <row r="41" spans="1:12">
       <c r="K41" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L41" s="15" t="s">
         <v>19</v>
-      </c>
-      <c r="L41" s="15" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:12">
       <c r="K42" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="L42" s="16" t="s">
         <v>21</v>
-      </c>
-      <c r="L42" s="16" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:12">
       <c r="K43" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="L43" s="15" t="s">
         <v>23</v>
-      </c>
-      <c r="L43" s="15" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="44" spans="1:12">
       <c r="K44" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="L44" s="15" t="s">
         <v>25</v>
-      </c>
-      <c r="L44" s="15" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="45" spans="1:12">
       <c r="K45" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L45" s="13"/>
     </row>
     <row r="46" spans="1:12">
       <c r="K46" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L46" s="13"/>
     </row>
     <row r="47" spans="1:12">
       <c r="K47" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L47" s="13"/>
     </row>
     <row r="48" spans="1:12">
       <c r="K48" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="L48" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="L48" s="15" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="49" spans="11:12">
       <c r="K49" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L49" s="13"/>
     </row>
     <row r="50" spans="11:12">
       <c r="K50" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="L50" s="18" t="s">
         <v>33</v>
-      </c>
-      <c r="L50" s="18" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="51" spans="11:12">
       <c r="K51" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L51" s="12" t="s">
         <v>35</v>
-      </c>
-      <c r="L51" s="12" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="52" spans="11:12">
       <c r="K52" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L52" s="12" t="s">
         <v>37</v>
-      </c>
-      <c r="L52" s="12" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="53" spans="11:12">
       <c r="K53" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="L53" s="12" t="s">
         <v>39</v>
-      </c>
-      <c r="L53" s="12" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="54" spans="11:12">
       <c r="K54" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L54" s="13"/>
     </row>
     <row r="55" spans="11:12">
       <c r="K55" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L55" s="13"/>
     </row>
     <row r="56" spans="11:12">
       <c r="K56" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="L56" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="L56" s="12" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="57" spans="11:12">
       <c r="K57" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="L57" s="12" t="s">
         <v>45</v>
-      </c>
-      <c r="L57" s="12" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="58" spans="11:12">
       <c r="K58" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L58" s="20"/>
     </row>
     <row r="59" spans="11:12">
       <c r="K59" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="L59" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="L59" s="12" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="60" spans="11:12">
       <c r="K60" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="L60" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="L60" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="61" spans="11:12">
       <c r="K61" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="L61" s="12" t="s">
         <v>52</v>
-      </c>
-      <c r="L61" s="12" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="62" spans="11:12">
       <c r="K62" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L62" s="20"/>
     </row>
     <row r="63" spans="11:12">
       <c r="K63" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="L63" s="12" t="s">
         <v>55</v>
-      </c>
-      <c r="L63" s="12" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="64" spans="11:12">
       <c r="K64" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="L64" s="12" t="s">
         <v>57</v>
-      </c>
-      <c r="L64" s="12" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="65" spans="1:12">
       <c r="K65" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L65" s="20"/>
     </row>
     <row r="66" spans="1:12">
       <c r="K66" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="L66" s="12" t="s">
         <v>60</v>
-      </c>
-      <c r="L66" s="12" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="67" spans="1:12">
       <c r="K67" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L67" s="13"/>
     </row>
     <row r="68" spans="1:12">
       <c r="K68" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L68" s="13"/>
     </row>
     <row r="69" spans="1:12">
       <c r="K69" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L69" s="13"/>
     </row>
     <row r="76" spans="1:12">
       <c r="A76" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2338,17 +2338,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0b19a164-5cac-4c2e-8d2c-1dd6255879dd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="14c5284c-9db7-464e-82e6-afebe603c4cc" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100964A9DE239497E4FB456E80342FF08E5" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="13c5b5de194996a54f63fc0ad6fef13c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0b19a164-5cac-4c2e-8d2c-1dd6255879dd" xmlns:ns3="14c5284c-9db7-464e-82e6-afebe603c4cc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f79d983150536d5712dc5d1dc928a0f" ns2:_="" ns3:_="">
     <xsd:import namespace="0b19a164-5cac-4c2e-8d2c-1dd6255879dd"/>
@@ -2597,6 +2586,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0b19a164-5cac-4c2e-8d2c-1dd6255879dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="14c5284c-9db7-464e-82e6-afebe603c4cc" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0BE85EB-F304-48FF-A10E-A28D46811FCF}">
   <ds:schemaRefs>
@@ -2606,17 +2606,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E31AB77-FF4F-4CD1-B466-3840D5840549}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0b19a164-5cac-4c2e-8d2c-1dd6255879dd"/>
-    <ds:schemaRef ds:uri="14c5284c-9db7-464e-82e6-afebe603c4cc"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D11E3069-3DCC-4890-B9DA-8C9AFC82600F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2633,4 +2622,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E31AB77-FF4F-4CD1-B466-3840D5840549}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0b19a164-5cac-4c2e-8d2c-1dd6255879dd"/>
+    <ds:schemaRef ds:uri="14c5284c-9db7-464e-82e6-afebe603c4cc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>